<commit_message>
Update company profile and financials for Garcia Tech; modify JSON and Excel outputs for data room simulator
</commit_message>
<xml_diff>
--- a/utils/data-room-simulator/output/ap_aging.xlsx
+++ b/utils/data-room-simulator/output/ap_aging.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP Aging" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AP Aging" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,17 +417,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>bucket</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
@@ -452,10 +440,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1583556.04</v>
+        <v>1573717.48</v>
       </c>
       <c r="C2" t="n">
-        <v>77.5</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="3">
@@ -465,10 +453,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>316862.35</v>
+        <v>263005.33</v>
       </c>
       <c r="C3" t="n">
-        <v>15.5</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +466,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>114282.61</v>
+        <v>107145.53</v>
       </c>
       <c r="C4" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="5">
@@ -491,10 +479,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>29552.93</v>
+        <v>43110.61</v>
       </c>
       <c r="C5" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="6">
@@ -517,7 +505,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2044253.93</v>
+        <v>1986978.94</v>
       </c>
       <c r="C7" t="n">
         <v>100</v>

</xml_diff>